<commit_message>
Added new RDF data schemes and visual schemes for education-table29-32, fixed XLSX spreadsheets for education-table29-31
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/education-table29.xlsx
+++ b/sources/table_normalization/xlsx/education-table29.xlsx
@@ -78,7 +78,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -88,12 +88,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -118,16 +112,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -695,7 +687,7 @@
       <c r="AA1" s="1">
         <v>24</v>
       </c>
-      <c r="AB1" s="4" t="s">
+      <c r="AB1" s="3" t="s">
         <v>3</v>
       </c>
     </row>
@@ -781,7 +773,7 @@
       <c r="AA2" s="2">
         <v>3</v>
       </c>
-      <c r="AB2" s="5">
+      <c r="AB2" s="2">
         <f t="shared" ref="AB2:AB34" si="0">SUM(D2:AA2)</f>
         <v>46</v>
       </c>
@@ -868,7 +860,7 @@
       <c r="AA3" s="2">
         <v>2</v>
       </c>
-      <c r="AB3" s="5">
+      <c r="AB3" s="2">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
@@ -955,7 +947,7 @@
       <c r="AA4" s="2">
         <v>4</v>
       </c>
-      <c r="AB4" s="5">
+      <c r="AB4" s="2">
         <f t="shared" si="0"/>
         <v>79</v>
       </c>
@@ -1042,7 +1034,7 @@
       <c r="AA5" s="2">
         <v>2</v>
       </c>
-      <c r="AB5" s="5">
+      <c r="AB5" s="2">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
@@ -1129,7 +1121,7 @@
       <c r="AA6" s="2">
         <v>3</v>
       </c>
-      <c r="AB6" s="5">
+      <c r="AB6" s="2">
         <f t="shared" si="0"/>
         <v>63</v>
       </c>
@@ -1216,7 +1208,7 @@
       <c r="AA7" s="2">
         <v>-1</v>
       </c>
-      <c r="AB7" s="5">
+      <c r="AB7" s="2">
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
@@ -1303,7 +1295,7 @@
       <c r="AA8" s="2">
         <v>3</v>
       </c>
-      <c r="AB8" s="5">
+      <c r="AB8" s="2">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
@@ -1390,7 +1382,7 @@
       <c r="AA9" s="2">
         <v>4</v>
       </c>
-      <c r="AB9" s="5">
+      <c r="AB9" s="2">
         <f t="shared" si="0"/>
         <v>73</v>
       </c>
@@ -1477,7 +1469,7 @@
       <c r="AA10" s="2">
         <v>1</v>
       </c>
-      <c r="AB10" s="5">
+      <c r="AB10" s="2">
         <f t="shared" si="0"/>
         <v>69</v>
       </c>
@@ -1564,7 +1556,7 @@
       <c r="AA11" s="2">
         <v>2</v>
       </c>
-      <c r="AB11" s="5">
+      <c r="AB11" s="2">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
@@ -1651,7 +1643,7 @@
       <c r="AA12" s="2">
         <v>4</v>
       </c>
-      <c r="AB12" s="5">
+      <c r="AB12" s="2">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
@@ -1738,7 +1730,7 @@
       <c r="AA13" s="2">
         <v>3</v>
       </c>
-      <c r="AB13" s="5">
+      <c r="AB13" s="2">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
@@ -1825,7 +1817,7 @@
       <c r="AA14" s="2">
         <v>2</v>
       </c>
-      <c r="AB14" s="5">
+      <c r="AB14" s="2">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
@@ -1912,7 +1904,7 @@
       <c r="AA15" s="2">
         <v>2</v>
       </c>
-      <c r="AB15" s="5">
+      <c r="AB15" s="2">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
@@ -1999,7 +1991,7 @@
       <c r="AA16" s="2">
         <v>0</v>
       </c>
-      <c r="AB16" s="5">
+      <c r="AB16" s="2">
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
@@ -2086,7 +2078,7 @@
       <c r="AA17" s="2">
         <v>4</v>
       </c>
-      <c r="AB17" s="5">
+      <c r="AB17" s="2">
         <f t="shared" si="0"/>
         <v>57</v>
       </c>
@@ -2173,7 +2165,7 @@
       <c r="AA18" s="2">
         <v>3</v>
       </c>
-      <c r="AB18" s="5">
+      <c r="AB18" s="2">
         <f t="shared" si="0"/>
         <v>61</v>
       </c>
@@ -2260,7 +2252,7 @@
       <c r="AA19" s="2">
         <v>0</v>
       </c>
-      <c r="AB19" s="5">
+      <c r="AB19" s="2">
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
@@ -2347,7 +2339,7 @@
       <c r="AA20" s="2">
         <v>3</v>
       </c>
-      <c r="AB20" s="5">
+      <c r="AB20" s="2">
         <f t="shared" si="0"/>
         <v>86</v>
       </c>
@@ -2434,7 +2426,7 @@
       <c r="AA21" s="2">
         <v>0</v>
       </c>
-      <c r="AB21" s="5">
+      <c r="AB21" s="2">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
@@ -2521,7 +2513,7 @@
       <c r="AA22" s="2">
         <v>4</v>
       </c>
-      <c r="AB22" s="5">
+      <c r="AB22" s="2">
         <f t="shared" si="0"/>
         <v>76</v>
       </c>
@@ -2608,7 +2600,7 @@
       <c r="AA23" s="2">
         <v>2</v>
       </c>
-      <c r="AB23" s="5">
+      <c r="AB23" s="2">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
@@ -2695,7 +2687,7 @@
       <c r="AA24" s="2">
         <v>4</v>
       </c>
-      <c r="AB24" s="5">
+      <c r="AB24" s="2">
         <f t="shared" si="0"/>
         <v>53</v>
       </c>
@@ -2782,7 +2774,7 @@
       <c r="AA25" s="2">
         <v>3</v>
       </c>
-      <c r="AB25" s="5">
+      <c r="AB25" s="2">
         <f t="shared" si="0"/>
         <v>71</v>
       </c>
@@ -2869,7 +2861,7 @@
       <c r="AA26" s="2">
         <v>2</v>
       </c>
-      <c r="AB26" s="5">
+      <c r="AB26" s="2">
         <f t="shared" si="0"/>
         <v>63</v>
       </c>
@@ -2956,7 +2948,7 @@
       <c r="AA27" s="2">
         <v>2</v>
       </c>
-      <c r="AB27" s="5">
+      <c r="AB27" s="2">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
@@ -3043,7 +3035,7 @@
       <c r="AA28" s="2">
         <v>4</v>
       </c>
-      <c r="AB28" s="5">
+      <c r="AB28" s="2">
         <f t="shared" si="0"/>
         <v>68</v>
       </c>
@@ -3130,7 +3122,7 @@
       <c r="AA29" s="2">
         <v>1</v>
       </c>
-      <c r="AB29" s="5">
+      <c r="AB29" s="2">
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
@@ -3217,7 +3209,7 @@
       <c r="AA30" s="2">
         <v>3</v>
       </c>
-      <c r="AB30" s="5">
+      <c r="AB30" s="2">
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
@@ -3304,7 +3296,7 @@
       <c r="AA31" s="2">
         <v>3</v>
       </c>
-      <c r="AB31" s="5">
+      <c r="AB31" s="2">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
@@ -3391,7 +3383,7 @@
       <c r="AA32" s="2">
         <v>0</v>
       </c>
-      <c r="AB32" s="5">
+      <c r="AB32" s="2">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
@@ -3478,7 +3470,7 @@
       <c r="AA33" s="2">
         <v>3</v>
       </c>
-      <c r="AB33" s="5">
+      <c r="AB33" s="2">
         <f t="shared" si="0"/>
         <v>67</v>
       </c>
@@ -3565,13 +3557,13 @@
       <c r="AA34" s="2">
         <v>3</v>
       </c>
-      <c r="AB34" s="5">
+      <c r="AB34" s="2">
         <f t="shared" si="0"/>
         <v>71</v>
       </c>
     </row>
     <row r="35" spans="1:28">
-      <c r="C35" s="6" t="s">
+      <c r="C35" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D35" s="2">
@@ -3672,7 +3664,7 @@
       </c>
     </row>
     <row r="36" spans="1:28">
-      <c r="C36" s="6" t="s">
+      <c r="C36" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D36" s="2">
@@ -3773,7 +3765,7 @@
       </c>
     </row>
     <row r="37" spans="1:28">
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D37" s="2">

</xml_diff>